<commit_message>
vault backup: 2022-12-14 22:33:56
</commit_message>
<xml_diff>
--- a/40EWR_DIGI/Digimatic_Tabelle.xlsx
+++ b/40EWR_DIGI/Digimatic_Tabelle.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_docs\notes\40EWR_DIGI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D45C3917-BB0F-4C6C-B7BA-F55C416A1720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5D08B27-DF04-40D5-A074-68F479B2256C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="975" yWindow="0" windowWidth="26535" windowHeight="15105" xr2:uid="{3E82B335-DAA8-4F32-B234-7C205CAED7F1}"/>
+    <workbookView xWindow="30930" yWindow="2325" windowWidth="28800" windowHeight="16755" xr2:uid="{3E82B335-DAA8-4F32-B234-7C205CAED7F1}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -20,23 +20,46 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>ks-desktop</author>
+  </authors>
+  <commentList>
+    <comment ref="A8" authorId="0" shapeId="0" xr:uid="{581E76A0-195A-47CF-8987-961B345E34E1}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>ks-desktop:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+3G familie</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="27">
   <si>
     <t>T1</t>
   </si>
@@ -111,13 +134,19 @@
   </si>
   <si>
     <t>stabil</t>
+  </si>
+  <si>
+    <t>C1200</t>
+  </si>
+  <si>
+    <t>Millimess Touch</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -146,6 +175,19 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -736,7 +778,7 @@
                   <c:v>110</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>600</c:v>
+                  <c:v>1.2</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>13</c:v>
@@ -822,7 +864,7 @@
                   <c:v>108</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>800</c:v>
+                  <c:v>1.2</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>13</c:v>
@@ -1662,15 +1704,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>100011</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>138112</xdr:rowOff>
+      <xdr:colOff>109536</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>71437</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>1476375</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:colOff>1485900</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1994,7 +2036,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB7BB66-4805-4278-960F-48ED31F9AF97}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB7BB66-4805-4278-960F-48ED31F9AF97}">
   <dimension ref="A1:P19"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2087,13 +2129,13 @@
         <v>7</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O3" s="6" t="s">
         <v>7</v>
@@ -2377,7 +2419,7 @@
         <v>110</v>
       </c>
       <c r="F11" s="2">
-        <v>600</v>
+        <v>1.2</v>
       </c>
       <c r="G11" s="2">
         <v>13</v>
@@ -2403,7 +2445,7 @@
         <v>108</v>
       </c>
       <c r="F12" s="2">
-        <v>800</v>
+        <v>1.2</v>
       </c>
       <c r="G12" s="2">
         <v>13</v>
@@ -2413,6 +2455,9 @@
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -2421,6 +2466,9 @@
       <c r="G13" s="2"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -2472,5 +2520,6 @@
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
   <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>